<commit_message>
changed model to solar pro IQ4_XS
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ollama-Lamarckvergence-14B-Q8_0/2025-02-19_15-18-16/efficiency.xlsx
+++ b/res/efficiency/pet-md/ollama-Lamarckvergence-14B-Q8_0/2025-02-19_15-18-16/efficiency.xlsx
@@ -8,16 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\llm-process-generation\res\efficiency\pet-md\ollama-Lamarckvergence-14B-Q8_0\2025-02-19_15-18-16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7319C6-449C-4724-A092-6F8DC554D53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC3D89B-5B9E-4062-9315-73EA6F1DDB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Stats" sheetId="1" r:id="rId1"/>
     <sheet name="Answer_Stats" sheetId="2" r:id="rId2"/>
     <sheet name="Error_Stats" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -561,6 +574,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>